<commit_message>
ui, overhead reduction from delay
</commit_message>
<xml_diff>
--- a/IO/test/test_ip.xlsx
+++ b/IO/test/test_ip.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21267" windowHeight="8019"/>
+    <workbookView windowWidth="21267" windowHeight="8019" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="40t-1" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="200">
   <si>
     <t>FMM INFRA MOBILE CRANE PERMIT TRACKER</t>
   </si>
@@ -317,7 +317,7 @@
     <t>LD#3 &amp; TSCR</t>
   </si>
   <si>
-    <t>Alice</t>
+    <t>NAME100</t>
   </si>
   <si>
     <t>P-1001</t>
@@ -326,13 +326,13 @@
     <t>OK</t>
   </si>
   <si>
-    <t>Bob</t>
+    <t>NAME101</t>
   </si>
   <si>
     <t>P-1002</t>
   </si>
   <si>
-    <t>Charlie</t>
+    <t>NAME102</t>
   </si>
   <si>
     <t>P-1003</t>
@@ -341,37 +341,37 @@
     <t>Delayed</t>
   </si>
   <si>
-    <t>David</t>
+    <t>NAME103</t>
   </si>
   <si>
     <t>P-1004</t>
   </si>
   <si>
-    <t>Eve</t>
+    <t>NAME104</t>
   </si>
   <si>
     <t>P-1005</t>
   </si>
   <si>
-    <t>Frank</t>
+    <t>NAME105</t>
   </si>
   <si>
     <t>P-1006</t>
   </si>
   <si>
-    <t>Grace</t>
+    <t>NAME106</t>
   </si>
   <si>
     <t>P-1007</t>
   </si>
   <si>
-    <t>Heidi</t>
+    <t>NAME107</t>
   </si>
   <si>
     <t>P-1008</t>
   </si>
   <si>
-    <t>Ivan</t>
+    <t>NAME108</t>
   </si>
   <si>
     <t>P-1009</t>
@@ -380,13 +380,19 @@
     <t>PP</t>
   </si>
   <si>
-    <t>Judy</t>
+    <t>NAME109</t>
   </si>
   <si>
     <t>P-1010</t>
   </si>
   <si>
+    <t>NAME110</t>
+  </si>
+  <si>
     <t>P-1011</t>
+  </si>
+  <si>
+    <t>NAME111</t>
   </si>
   <si>
     <t>P-1012</t>
@@ -395,58 +401,115 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
+    <t>NAME112</t>
+  </si>
+  <si>
     <t>P-1013</t>
+  </si>
+  <si>
+    <t>NAME113</t>
   </si>
   <si>
     <t>P-1014</t>
   </si>
   <si>
+    <t>NAME114</t>
+  </si>
+  <si>
     <t>P-1015</t>
+  </si>
+  <si>
+    <t>NAME115</t>
   </si>
   <si>
     <t>P-1016</t>
   </si>
   <si>
+    <t>NAME116</t>
+  </si>
+  <si>
     <t>P-1017</t>
+  </si>
+  <si>
+    <t>NAME117</t>
   </si>
   <si>
     <t>P-1018</t>
   </si>
   <si>
+    <t>NAME118</t>
+  </si>
+  <si>
     <t>P-1019</t>
+  </si>
+  <si>
+    <t>NAME119</t>
   </si>
   <si>
     <t>P-1020</t>
   </si>
   <si>
+    <t>NAME120</t>
+  </si>
+  <si>
     <t>P-1021</t>
+  </si>
+  <si>
+    <t>NAME121</t>
   </si>
   <si>
     <t>P-1022</t>
   </si>
   <si>
+    <t>NAME122</t>
+  </si>
+  <si>
     <t>P-1023</t>
+  </si>
+  <si>
+    <t>NAME123</t>
   </si>
   <si>
     <t>P-1024</t>
   </si>
   <si>
+    <t>NAME124</t>
+  </si>
+  <si>
     <t>P-1025</t>
+  </si>
+  <si>
+    <t>NAME125</t>
   </si>
   <si>
     <t>P-1026</t>
   </si>
   <si>
+    <t>NAME126</t>
+  </si>
+  <si>
     <t>P-1027</t>
+  </si>
+  <si>
+    <t>NAME127</t>
   </si>
   <si>
     <t>P-1028</t>
   </si>
   <si>
+    <t>NAME128</t>
+  </si>
+  <si>
     <t>P-1029</t>
   </si>
   <si>
+    <t>NAME129</t>
+  </si>
+  <si>
     <t>P-1030</t>
+  </si>
+  <si>
+    <t>NAME130</t>
   </si>
   <si>
     <t>P-1031</t>
@@ -458,13 +521,106 @@
     <t>HP38F-9542</t>
   </si>
   <si>
+    <t>NAME300</t>
+  </si>
+  <si>
+    <t>NAME301</t>
+  </si>
+  <si>
+    <t>NAME302</t>
+  </si>
+  <si>
     <t>CRM</t>
+  </si>
+  <si>
+    <t>NAME303</t>
+  </si>
+  <si>
+    <t>NAME304</t>
+  </si>
+  <si>
+    <t>NAME305</t>
+  </si>
+  <si>
+    <t>NAME306</t>
+  </si>
+  <si>
+    <t>NAME307</t>
+  </si>
+  <si>
+    <t>NAME308</t>
   </si>
   <si>
     <t>LP</t>
   </si>
   <si>
+    <t>NAME309</t>
+  </si>
+  <si>
+    <t>NAME310</t>
+  </si>
+  <si>
+    <t>NAME311</t>
+  </si>
+  <si>
+    <t>NAME312</t>
+  </si>
+  <si>
+    <t>NAME313</t>
+  </si>
+  <si>
+    <t>NAME314</t>
+  </si>
+  <si>
+    <t>NAME315</t>
+  </si>
+  <si>
+    <t>NAME316</t>
+  </si>
+  <si>
+    <t>NAME317</t>
+  </si>
+  <si>
+    <t>NAME318</t>
+  </si>
+  <si>
+    <t>NAME319</t>
+  </si>
+  <si>
+    <t>NAME320</t>
+  </si>
+  <si>
+    <t>NAME321</t>
+  </si>
+  <si>
+    <t>NAME322</t>
+  </si>
+  <si>
+    <t>NAME323</t>
+  </si>
+  <si>
+    <t>NAME324</t>
+  </si>
+  <si>
     <t>IBF</t>
+  </si>
+  <si>
+    <t>NAME325</t>
+  </si>
+  <si>
+    <t>NAME326</t>
+  </si>
+  <si>
+    <t>NAME327</t>
+  </si>
+  <si>
+    <t>NAME328</t>
+  </si>
+  <si>
+    <t>NAME329</t>
+  </si>
+  <si>
+    <t>NAME330</t>
   </si>
   <si>
     <t>CRANE :- 300T-1</t>
@@ -30003,7 +30159,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" ht="14.4" spans="1:10">
+    <row r="4" spans="1:10">
       <c r="A4" s="62">
         <v>1</v>
       </c>
@@ -30048,7 +30204,7 @@
       <c r="D5" s="64" t="s">
         <v>41</v>
       </c>
-      <c r="E5" s="64" t="s">
+      <c r="E5" s="62" t="s">
         <v>98</v>
       </c>
       <c r="F5" s="69">
@@ -30081,7 +30237,7 @@
       <c r="D6" s="64" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="64" t="s">
+      <c r="E6" s="62" t="s">
         <v>100</v>
       </c>
       <c r="F6" s="64">
@@ -30101,7 +30257,7 @@
       </c>
       <c r="O6" s="44"/>
     </row>
-    <row r="7" ht="14.4" spans="1:10">
+    <row r="7" spans="1:10">
       <c r="A7" s="62">
         <v>4</v>
       </c>
@@ -30114,7 +30270,7 @@
       <c r="D7" s="64" t="s">
         <v>94</v>
       </c>
-      <c r="E7" s="72" t="s">
+      <c r="E7" s="62" t="s">
         <v>103</v>
       </c>
       <c r="F7" s="72">
@@ -30146,7 +30302,7 @@
       <c r="D8" s="64" t="s">
         <v>51</v>
       </c>
-      <c r="E8" s="72" t="s">
+      <c r="E8" s="62" t="s">
         <v>105</v>
       </c>
       <c r="F8" s="72">
@@ -30166,7 +30322,7 @@
       </c>
       <c r="Q8" s="52"/>
     </row>
-    <row r="9" ht="14.4" spans="1:10">
+    <row r="9" spans="1:10">
       <c r="A9" s="62">
         <v>6</v>
       </c>
@@ -30179,7 +30335,7 @@
       <c r="D9" s="64" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="72" t="s">
+      <c r="E9" s="62" t="s">
         <v>107</v>
       </c>
       <c r="F9" s="72">
@@ -30211,7 +30367,7 @@
       <c r="D10" s="64" t="s">
         <v>46</v>
       </c>
-      <c r="E10" s="72" t="s">
+      <c r="E10" s="62" t="s">
         <v>109</v>
       </c>
       <c r="F10" s="72">
@@ -30245,7 +30401,7 @@
       <c r="D11" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="72" t="s">
+      <c r="E11" s="62" t="s">
         <v>111</v>
       </c>
       <c r="F11" s="72">
@@ -30278,7 +30434,7 @@
       <c r="D12" s="64" t="s">
         <v>30</v>
       </c>
-      <c r="E12" s="72" t="s">
+      <c r="E12" s="62" t="s">
         <v>113</v>
       </c>
       <c r="F12" s="72">
@@ -30311,7 +30467,7 @@
       <c r="D13" s="64" t="s">
         <v>115</v>
       </c>
-      <c r="E13" s="72" t="s">
+      <c r="E13" s="62" t="s">
         <v>116</v>
       </c>
       <c r="F13" s="72">
@@ -30344,8 +30500,8 @@
       <c r="D14" s="64" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="72" t="s">
-        <v>95</v>
+      <c r="E14" s="62" t="s">
+        <v>118</v>
       </c>
       <c r="F14" s="72">
         <v>9876543210</v>
@@ -30354,7 +30510,7 @@
         <v>0.364583333333333</v>
       </c>
       <c r="H14" s="71" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I14" s="70">
         <v>0.510416666666667</v>
@@ -30377,8 +30533,8 @@
       <c r="D15" s="64" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="72" t="s">
-        <v>98</v>
+      <c r="E15" s="62" t="s">
+        <v>120</v>
       </c>
       <c r="F15" s="72">
         <v>9876543211</v>
@@ -30387,7 +30543,7 @@
         <v>0.385416666666667</v>
       </c>
       <c r="H15" s="71" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="I15" s="70">
         <v>0.489583333333333</v>
@@ -30396,7 +30552,7 @@
         <v>97</v>
       </c>
       <c r="K15" s="50" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="O15" s="44"/>
     </row>
@@ -30413,8 +30569,8 @@
       <c r="D16" s="64" t="s">
         <v>63</v>
       </c>
-      <c r="E16" s="72" t="s">
-        <v>100</v>
+      <c r="E16" s="62" t="s">
+        <v>123</v>
       </c>
       <c r="F16" s="72">
         <v>9876543212</v>
@@ -30423,7 +30579,7 @@
         <v>0.4375</v>
       </c>
       <c r="H16" s="71" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I16" s="70">
         <v>0.583333333333333</v>
@@ -30446,8 +30602,8 @@
       <c r="D17" s="64" t="s">
         <v>38</v>
       </c>
-      <c r="E17" s="72" t="s">
-        <v>103</v>
+      <c r="E17" s="62" t="s">
+        <v>125</v>
       </c>
       <c r="F17" s="72">
         <v>9876543213</v>
@@ -30456,7 +30612,7 @@
         <v>0.333333333333333</v>
       </c>
       <c r="H17" s="71" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="I17" s="70">
         <v>0.416666666666667</v>
@@ -30479,8 +30635,8 @@
       <c r="D18" s="64" t="s">
         <v>115</v>
       </c>
-      <c r="E18" s="72" t="s">
-        <v>105</v>
+      <c r="E18" s="62" t="s">
+        <v>127</v>
       </c>
       <c r="F18" s="72">
         <v>9876543214</v>
@@ -30489,7 +30645,7 @@
         <v>0.40625</v>
       </c>
       <c r="H18" s="71" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="I18" s="70">
         <v>0.552083333333333</v>
@@ -30499,7 +30655,7 @@
       </c>
       <c r="N18" s="52"/>
     </row>
-    <row r="19" ht="14.4" spans="1:10">
+    <row r="19" spans="1:10">
       <c r="A19" s="62">
         <v>16</v>
       </c>
@@ -30512,8 +30668,8 @@
       <c r="D19" s="64" t="s">
         <v>17</v>
       </c>
-      <c r="E19" s="72" t="s">
-        <v>107</v>
+      <c r="E19" s="62" t="s">
+        <v>129</v>
       </c>
       <c r="F19" s="72">
         <v>9876543215</v>
@@ -30522,7 +30678,7 @@
         <v>0.354166666666667</v>
       </c>
       <c r="H19" s="71" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="I19" s="70">
         <v>0.479166666666667</v>
@@ -30531,7 +30687,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="20" ht="14.4" spans="1:10">
+    <row r="20" spans="1:10">
       <c r="A20" s="62">
         <v>17</v>
       </c>
@@ -30544,8 +30700,8 @@
       <c r="D20" s="64" t="s">
         <v>30</v>
       </c>
-      <c r="E20" s="72" t="s">
-        <v>109</v>
+      <c r="E20" s="62" t="s">
+        <v>131</v>
       </c>
       <c r="F20" s="72">
         <v>9876543216</v>
@@ -30554,7 +30710,7 @@
         <v>0.416666666666667</v>
       </c>
       <c r="H20" s="71" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="I20" s="70">
         <v>0.520833333333333</v>
@@ -30563,7 +30719,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="21" ht="14.4" spans="1:10">
+    <row r="21" spans="1:10">
       <c r="A21" s="62">
         <v>18</v>
       </c>
@@ -30576,8 +30732,8 @@
       <c r="D21" s="64" t="s">
         <v>115</v>
       </c>
-      <c r="E21" s="72" t="s">
-        <v>111</v>
+      <c r="E21" s="62" t="s">
+        <v>133</v>
       </c>
       <c r="F21" s="72">
         <v>9876543217</v>
@@ -30586,7 +30742,7 @@
         <v>0.322916666666667</v>
       </c>
       <c r="H21" s="71" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="I21" s="70">
         <v>0.40625</v>
@@ -30595,7 +30751,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="22" ht="14.4" spans="1:10">
+    <row r="22" spans="1:10">
       <c r="A22" s="62">
         <v>19</v>
       </c>
@@ -30608,8 +30764,8 @@
       <c r="D22" s="64" t="s">
         <v>21</v>
       </c>
-      <c r="E22" s="72" t="s">
-        <v>113</v>
+      <c r="E22" s="62" t="s">
+        <v>135</v>
       </c>
       <c r="F22" s="72">
         <v>9876543218</v>
@@ -30618,7 +30774,7 @@
         <v>0.34375</v>
       </c>
       <c r="H22" s="71" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="I22" s="70">
         <v>0.447916666666667</v>
@@ -30627,7 +30783,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="23" ht="14.4" spans="1:10">
+    <row r="23" spans="1:10">
       <c r="A23" s="62">
         <v>20</v>
       </c>
@@ -30640,8 +30796,8 @@
       <c r="D23" s="64" t="s">
         <v>41</v>
       </c>
-      <c r="E23" s="72" t="s">
-        <v>116</v>
+      <c r="E23" s="62" t="s">
+        <v>137</v>
       </c>
       <c r="F23" s="72">
         <v>9876543219</v>
@@ -30650,7 +30806,7 @@
         <v>0.375</v>
       </c>
       <c r="H23" s="71" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I23" s="70">
         <v>0.458333333333333</v>
@@ -30659,7 +30815,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="24" ht="14.4" spans="1:10">
+    <row r="24" spans="1:10">
       <c r="A24" s="62">
         <v>21</v>
       </c>
@@ -30672,8 +30828,8 @@
       <c r="D24" s="64" t="s">
         <v>21</v>
       </c>
-      <c r="E24" s="72" t="s">
-        <v>95</v>
+      <c r="E24" s="62" t="s">
+        <v>139</v>
       </c>
       <c r="F24" s="72">
         <v>9876543210</v>
@@ -30682,7 +30838,7 @@
         <v>0.427083333333333</v>
       </c>
       <c r="H24" s="71" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="I24" s="70">
         <v>0.59375</v>
@@ -30691,7 +30847,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="25" ht="14.4" spans="1:10">
+    <row r="25" spans="1:10">
       <c r="A25" s="62">
         <v>22</v>
       </c>
@@ -30704,8 +30860,8 @@
       <c r="D25" s="64" t="s">
         <v>115</v>
       </c>
-      <c r="E25" s="72" t="s">
-        <v>98</v>
+      <c r="E25" s="62" t="s">
+        <v>141</v>
       </c>
       <c r="F25" s="72">
         <v>9876543211</v>
@@ -30714,7 +30870,7 @@
         <v>0.333333333333333</v>
       </c>
       <c r="H25" s="71" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="I25" s="70">
         <v>0.4375</v>
@@ -30723,7 +30879,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="26" ht="14.4" spans="1:10">
+    <row r="26" spans="1:10">
       <c r="A26" s="62">
         <v>23</v>
       </c>
@@ -30736,8 +30892,8 @@
       <c r="D26" s="64" t="s">
         <v>115</v>
       </c>
-      <c r="E26" s="72" t="s">
-        <v>100</v>
+      <c r="E26" s="62" t="s">
+        <v>143</v>
       </c>
       <c r="F26" s="72">
         <v>9876543212</v>
@@ -30746,7 +30902,7 @@
         <v>0.395833333333333</v>
       </c>
       <c r="H26" s="71" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="I26" s="70">
         <v>0.5</v>
@@ -30755,7 +30911,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="27" ht="14.4" spans="1:10">
+    <row r="27" spans="1:10">
       <c r="A27" s="62">
         <v>24</v>
       </c>
@@ -30768,8 +30924,8 @@
       <c r="D27" s="64" t="s">
         <v>33</v>
       </c>
-      <c r="E27" s="72" t="s">
-        <v>103</v>
+      <c r="E27" s="62" t="s">
+        <v>145</v>
       </c>
       <c r="F27" s="72">
         <v>9876543213</v>
@@ -30778,7 +30934,7 @@
         <v>0.364583333333333</v>
       </c>
       <c r="H27" s="71" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="I27" s="70">
         <v>0.46875</v>
@@ -30787,7 +30943,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="28" ht="14.4" spans="1:10">
+    <row r="28" spans="1:10">
       <c r="A28" s="62">
         <v>25</v>
       </c>
@@ -30800,8 +30956,8 @@
       <c r="D28" s="64" t="s">
         <v>30</v>
       </c>
-      <c r="E28" s="64" t="s">
-        <v>105</v>
+      <c r="E28" s="62" t="s">
+        <v>147</v>
       </c>
       <c r="F28" s="69">
         <v>9876543214</v>
@@ -30810,7 +30966,7 @@
         <v>0.3125</v>
       </c>
       <c r="H28" s="71" t="s">
-        <v>133</v>
+        <v>148</v>
       </c>
       <c r="I28" s="70">
         <v>0.395833333333333</v>
@@ -30819,7 +30975,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="29" ht="14.4" spans="1:10">
+    <row r="29" spans="1:10">
       <c r="A29" s="62">
         <v>26</v>
       </c>
@@ -30832,8 +30988,8 @@
       <c r="D29" s="64" t="s">
         <v>33</v>
       </c>
-      <c r="E29" s="72" t="s">
-        <v>107</v>
+      <c r="E29" s="62" t="s">
+        <v>149</v>
       </c>
       <c r="F29" s="72">
         <v>9876543215</v>
@@ -30842,7 +30998,7 @@
         <v>0.416666666666667</v>
       </c>
       <c r="H29" s="71" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="I29" s="70">
         <v>0.541666666666667</v>
@@ -30851,7 +31007,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="30" ht="14.4" spans="1:10">
+    <row r="30" spans="1:10">
       <c r="A30" s="62">
         <v>27</v>
       </c>
@@ -30864,8 +31020,8 @@
       <c r="D30" s="64" t="s">
         <v>30</v>
       </c>
-      <c r="E30" s="72" t="s">
-        <v>109</v>
+      <c r="E30" s="62" t="s">
+        <v>151</v>
       </c>
       <c r="F30" s="72">
         <v>9876543216</v>
@@ -30874,7 +31030,7 @@
         <v>0.34375</v>
       </c>
       <c r="H30" s="71" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
       <c r="I30" s="70">
         <v>0.489583333333333</v>
@@ -30883,7 +31039,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="31" ht="14.4" spans="1:10">
+    <row r="31" spans="1:10">
       <c r="A31" s="62">
         <v>28</v>
       </c>
@@ -30896,8 +31052,8 @@
       <c r="D31" s="64" t="s">
         <v>38</v>
       </c>
-      <c r="E31" s="64" t="s">
-        <v>111</v>
+      <c r="E31" s="62" t="s">
+        <v>153</v>
       </c>
       <c r="F31" s="69">
         <v>9876543217</v>
@@ -30906,7 +31062,7 @@
         <v>0.375</v>
       </c>
       <c r="H31" s="71" t="s">
-        <v>136</v>
+        <v>154</v>
       </c>
       <c r="I31" s="70">
         <v>0.520833333333333</v>
@@ -30915,7 +31071,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="32" ht="14.4" spans="1:10">
+    <row r="32" spans="1:10">
       <c r="A32" s="62">
         <v>29</v>
       </c>
@@ -30928,8 +31084,8 @@
       <c r="D32" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="E32" s="65" t="s">
-        <v>113</v>
+      <c r="E32" s="62" t="s">
+        <v>155</v>
       </c>
       <c r="F32" s="65">
         <v>9876543218</v>
@@ -30938,7 +31094,7 @@
         <v>0.354166666666667</v>
       </c>
       <c r="H32" s="65" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="I32" s="66">
         <v>0.4375</v>
@@ -30947,7 +31103,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="33" ht="14.4" spans="1:10">
+    <row r="33" spans="1:10">
       <c r="A33" s="62">
         <v>30</v>
       </c>
@@ -30960,8 +31116,8 @@
       <c r="D33" s="65" t="s">
         <v>30</v>
       </c>
-      <c r="E33" s="65" t="s">
-        <v>116</v>
+      <c r="E33" s="62" t="s">
+        <v>157</v>
       </c>
       <c r="F33" s="65">
         <v>9876543219</v>
@@ -30970,7 +31126,7 @@
         <v>0.447916666666667</v>
       </c>
       <c r="H33" s="65" t="s">
-        <v>138</v>
+        <v>158</v>
       </c>
       <c r="I33" s="66">
         <v>0.625</v>
@@ -30979,7 +31135,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="34" ht="14.4" spans="1:10">
+    <row r="34" spans="1:10">
       <c r="A34" s="62">
         <v>31</v>
       </c>
@@ -30992,8 +31148,8 @@
       <c r="D34" s="65" t="s">
         <v>46</v>
       </c>
-      <c r="E34" s="65" t="s">
-        <v>95</v>
+      <c r="E34" s="62" t="s">
+        <v>159</v>
       </c>
       <c r="F34" s="65">
         <v>9876543210</v>
@@ -31002,7 +31158,7 @@
         <v>0.385416666666667</v>
       </c>
       <c r="H34" s="65" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="I34" s="66">
         <v>0.46875</v>
@@ -42663,7 +42819,7 @@
       <c r="D2" s="5"/>
       <c r="E2" s="6"/>
       <c r="F2" s="7" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
       <c r="G2" s="8"/>
       <c r="H2" s="9" t="s">
@@ -42706,7 +42862,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" ht="14.4" spans="1:10">
+    <row r="4" spans="1:10">
       <c r="A4" s="15">
         <v>1</v>
       </c>
@@ -42714,12 +42870,14 @@
         <v>46082</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D4" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="E4" s="17"/>
+      <c r="E4" s="17" t="s">
+        <v>163</v>
+      </c>
       <c r="F4" s="19"/>
       <c r="G4" s="40">
         <v>0.724305555555556</v>
@@ -42738,12 +42896,14 @@
         <v>46083</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D5" s="39" t="s">
         <v>94</v>
       </c>
-      <c r="E5" s="39"/>
+      <c r="E5" s="17" t="s">
+        <v>164</v>
+      </c>
       <c r="F5" s="23"/>
       <c r="G5" s="41">
         <v>0.431944444444444</v>
@@ -42763,12 +42923,14 @@
         <v>46084</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D6" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="E6" s="25"/>
+      <c r="E6" s="17" t="s">
+        <v>165</v>
+      </c>
       <c r="F6" s="25"/>
       <c r="G6" s="42">
         <v>0.629861111111111</v>
@@ -42780,7 +42942,7 @@
       <c r="J6" s="35"/>
       <c r="O6" s="44"/>
     </row>
-    <row r="7" ht="14.4" spans="1:10">
+    <row r="7" spans="1:10">
       <c r="A7" s="15">
         <v>4</v>
       </c>
@@ -42788,12 +42950,14 @@
         <v>46085</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D7" s="39" t="s">
-        <v>142</v>
-      </c>
-      <c r="E7" s="27"/>
+        <v>166</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>167</v>
+      </c>
       <c r="F7" s="27"/>
       <c r="G7" s="41">
         <v>0.638888888888889</v>
@@ -42812,12 +42976,14 @@
         <v>46086</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D8" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="27"/>
+      <c r="E8" s="17" t="s">
+        <v>168</v>
+      </c>
       <c r="F8" s="27"/>
       <c r="G8" s="41">
         <v>0.448611111111111</v>
@@ -42829,7 +42995,7 @@
       <c r="J8" s="34"/>
       <c r="Q8" s="52"/>
     </row>
-    <row r="9" ht="14.4" spans="1:10">
+    <row r="9" spans="1:10">
       <c r="A9" s="15">
         <v>6</v>
       </c>
@@ -42837,12 +43003,14 @@
         <v>46087</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D9" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="E9" s="27"/>
+      <c r="E9" s="17" t="s">
+        <v>169</v>
+      </c>
       <c r="F9" s="27"/>
       <c r="G9" s="41">
         <v>0.265972222222222</v>
@@ -42861,12 +43029,14 @@
         <v>46088</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D10" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="27"/>
+      <c r="E10" s="17" t="s">
+        <v>170</v>
+      </c>
       <c r="F10" s="27"/>
       <c r="G10" s="41">
         <v>0.59375</v>
@@ -42887,12 +43057,14 @@
         <v>46089</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D11" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="27"/>
+      <c r="E11" s="17" t="s">
+        <v>171</v>
+      </c>
       <c r="F11" s="27"/>
       <c r="G11" s="41">
         <v>0.698611111111111</v>
@@ -42912,12 +43084,14 @@
         <v>46090</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D12" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="E12" s="27"/>
+      <c r="E12" s="17" t="s">
+        <v>172</v>
+      </c>
       <c r="F12" s="27"/>
       <c r="G12" s="41">
         <v>0.545138888888889</v>
@@ -42937,12 +43111,14 @@
         <v>46091</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D13" s="39" t="s">
-        <v>143</v>
-      </c>
-      <c r="E13" s="27"/>
+        <v>173</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>174</v>
+      </c>
       <c r="F13" s="27"/>
       <c r="G13" s="41">
         <v>0.286111111111111</v>
@@ -42962,12 +43138,14 @@
         <v>46092</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D14" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="27"/>
+      <c r="E14" s="17" t="s">
+        <v>175</v>
+      </c>
       <c r="F14" s="27"/>
       <c r="G14" s="41">
         <v>0.340277777777778</v>
@@ -42987,12 +43165,14 @@
         <v>46093</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D15" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="27"/>
+      <c r="E15" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="F15" s="27"/>
       <c r="G15" s="41">
         <v>0.281944444444444</v>
@@ -43003,7 +43183,7 @@
       </c>
       <c r="J15" s="34"/>
       <c r="K15" s="50" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="O15" s="44"/>
     </row>
@@ -43015,12 +43195,14 @@
         <v>46094</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D16" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="E16" s="27"/>
+      <c r="E16" s="17" t="s">
+        <v>177</v>
+      </c>
       <c r="F16" s="27"/>
       <c r="G16" s="41">
         <v>0.6125</v>
@@ -43040,12 +43222,14 @@
         <v>46095</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D17" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="E17" s="27"/>
+      <c r="E17" s="17" t="s">
+        <v>178</v>
+      </c>
       <c r="F17" s="27"/>
       <c r="G17" s="41">
         <v>0.649305555555556</v>
@@ -43065,12 +43249,14 @@
         <v>46096</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D18" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="E18" s="27"/>
+      <c r="E18" s="17" t="s">
+        <v>179</v>
+      </c>
       <c r="F18" s="27"/>
       <c r="G18" s="41">
         <v>0.717361111111111</v>
@@ -43082,7 +43268,7 @@
       <c r="J18" s="34"/>
       <c r="N18" s="52"/>
     </row>
-    <row r="19" ht="14.4" spans="1:10">
+    <row r="19" spans="1:10">
       <c r="A19" s="15">
         <v>16</v>
       </c>
@@ -43090,12 +43276,14 @@
         <v>46097</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D19" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="27"/>
+      <c r="E19" s="17" t="s">
+        <v>180</v>
+      </c>
       <c r="F19" s="27"/>
       <c r="G19" s="41">
         <v>0.609722222222222</v>
@@ -43106,7 +43294,7 @@
       </c>
       <c r="J19" s="34"/>
     </row>
-    <row r="20" ht="14.4" spans="1:10">
+    <row r="20" spans="1:10">
       <c r="A20" s="15">
         <v>17</v>
       </c>
@@ -43114,12 +43302,14 @@
         <v>46098</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D20" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="E20" s="27"/>
+      <c r="E20" s="17" t="s">
+        <v>181</v>
+      </c>
       <c r="F20" s="27"/>
       <c r="G20" s="41">
         <v>0.615972222222222</v>
@@ -43130,7 +43320,7 @@
       </c>
       <c r="J20" s="34"/>
     </row>
-    <row r="21" ht="14.4" spans="1:10">
+    <row r="21" spans="1:10">
       <c r="A21" s="15">
         <v>18</v>
       </c>
@@ -43138,12 +43328,14 @@
         <v>46099</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D21" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="E21" s="27"/>
+      <c r="E21" s="17" t="s">
+        <v>182</v>
+      </c>
       <c r="F21" s="27"/>
       <c r="G21" s="41">
         <v>0.660416666666667</v>
@@ -43154,7 +43346,7 @@
       </c>
       <c r="J21" s="34"/>
     </row>
-    <row r="22" ht="14.4" spans="1:10">
+    <row r="22" spans="1:10">
       <c r="A22" s="15">
         <v>19</v>
       </c>
@@ -43162,12 +43354,14 @@
         <v>46100</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D22" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="E22" s="27"/>
+      <c r="E22" s="17" t="s">
+        <v>183</v>
+      </c>
       <c r="F22" s="27"/>
       <c r="G22" s="41">
         <v>0.74375</v>
@@ -43178,7 +43372,7 @@
       </c>
       <c r="J22" s="34"/>
     </row>
-    <row r="23" ht="14.4" spans="1:10">
+    <row r="23" spans="1:10">
       <c r="A23" s="15">
         <v>20</v>
       </c>
@@ -43186,12 +43380,14 @@
         <v>46101</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D23" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="E23" s="27"/>
+      <c r="E23" s="17" t="s">
+        <v>184</v>
+      </c>
       <c r="F23" s="27"/>
       <c r="G23" s="41">
         <v>0.286805555555556</v>
@@ -43202,7 +43398,7 @@
       </c>
       <c r="J23" s="34"/>
     </row>
-    <row r="24" ht="14.4" spans="1:10">
+    <row r="24" spans="1:10">
       <c r="A24" s="15">
         <v>21</v>
       </c>
@@ -43210,12 +43406,14 @@
         <v>46102</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D24" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="E24" s="27"/>
+      <c r="E24" s="17" t="s">
+        <v>185</v>
+      </c>
       <c r="F24" s="27"/>
       <c r="G24" s="41">
         <v>0.478472222222222</v>
@@ -43226,7 +43424,7 @@
       </c>
       <c r="J24" s="34"/>
     </row>
-    <row r="25" ht="14.4" spans="1:10">
+    <row r="25" spans="1:10">
       <c r="A25" s="15">
         <v>22</v>
       </c>
@@ -43234,12 +43432,14 @@
         <v>46103</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D25" s="39" t="s">
         <v>56</v>
       </c>
-      <c r="E25" s="27"/>
+      <c r="E25" s="17" t="s">
+        <v>186</v>
+      </c>
       <c r="F25" s="27"/>
       <c r="G25" s="41">
         <v>0.386111111111111</v>
@@ -43250,7 +43450,7 @@
       </c>
       <c r="J25" s="34"/>
     </row>
-    <row r="26" ht="14.4" spans="1:10">
+    <row r="26" spans="1:10">
       <c r="A26" s="15">
         <v>23</v>
       </c>
@@ -43258,12 +43458,14 @@
         <v>46104</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D26" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="E26" s="27"/>
+      <c r="E26" s="17" t="s">
+        <v>187</v>
+      </c>
       <c r="F26" s="27"/>
       <c r="G26" s="41">
         <v>0.6125</v>
@@ -43274,7 +43476,7 @@
       </c>
       <c r="J26" s="34"/>
     </row>
-    <row r="27" ht="14.4" spans="1:10">
+    <row r="27" spans="1:10">
       <c r="A27" s="15">
         <v>24</v>
       </c>
@@ -43282,12 +43484,14 @@
         <v>46105</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D27" s="39" t="s">
         <v>63</v>
       </c>
-      <c r="E27" s="27"/>
+      <c r="E27" s="17" t="s">
+        <v>188</v>
+      </c>
       <c r="F27" s="27"/>
       <c r="G27" s="41">
         <v>0.765972222222222</v>
@@ -43298,7 +43502,7 @@
       </c>
       <c r="J27" s="34"/>
     </row>
-    <row r="28" ht="14.4" spans="1:10">
+    <row r="28" spans="1:10">
       <c r="A28" s="15">
         <v>25</v>
       </c>
@@ -43306,12 +43510,14 @@
         <v>46106</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D28" s="39" t="s">
-        <v>142</v>
-      </c>
-      <c r="E28" s="39"/>
+        <v>166</v>
+      </c>
+      <c r="E28" s="17" t="s">
+        <v>189</v>
+      </c>
       <c r="F28" s="23"/>
       <c r="G28" s="41">
         <v>0.452777777777778</v>
@@ -43322,7 +43528,7 @@
       </c>
       <c r="J28" s="34"/>
     </row>
-    <row r="29" ht="14.4" spans="1:10">
+    <row r="29" spans="1:10">
       <c r="A29" s="15">
         <v>26</v>
       </c>
@@ -43330,12 +43536,14 @@
         <v>46107</v>
       </c>
       <c r="C29" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D29" s="39" t="s">
-        <v>144</v>
-      </c>
-      <c r="E29" s="27"/>
+        <v>190</v>
+      </c>
+      <c r="E29" s="17" t="s">
+        <v>191</v>
+      </c>
       <c r="F29" s="27"/>
       <c r="G29" s="41">
         <v>0.339583333333333</v>
@@ -43346,7 +43554,7 @@
       </c>
       <c r="J29" s="34"/>
     </row>
-    <row r="30" ht="14.4" spans="1:10">
+    <row r="30" spans="1:10">
       <c r="A30" s="15">
         <v>27</v>
       </c>
@@ -43354,12 +43562,14 @@
         <v>46108</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D30" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="E30" s="27"/>
+      <c r="E30" s="17" t="s">
+        <v>192</v>
+      </c>
       <c r="F30" s="27"/>
       <c r="G30" s="41">
         <v>0.485416666666667</v>
@@ -43370,7 +43580,7 @@
       </c>
       <c r="J30" s="34"/>
     </row>
-    <row r="31" ht="14.4" spans="1:10">
+    <row r="31" spans="1:10">
       <c r="A31" s="15">
         <v>28</v>
       </c>
@@ -43378,12 +43588,14 @@
         <v>46109</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D31" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="E31" s="39"/>
+      <c r="E31" s="17" t="s">
+        <v>193</v>
+      </c>
       <c r="F31" s="23"/>
       <c r="G31" s="41">
         <v>0.782638888888889</v>
@@ -43394,7 +43606,7 @@
       </c>
       <c r="J31" s="34"/>
     </row>
-    <row r="32" ht="14.4" spans="1:10">
+    <row r="32" spans="1:10">
       <c r="A32" s="15">
         <v>29</v>
       </c>
@@ -43402,12 +43614,14 @@
         <v>46110</v>
       </c>
       <c r="C32" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D32" s="19" t="s">
-        <v>142</v>
-      </c>
-      <c r="E32" s="19"/>
+        <v>166</v>
+      </c>
+      <c r="E32" s="17" t="s">
+        <v>194</v>
+      </c>
       <c r="F32" s="19"/>
       <c r="G32" s="40">
         <v>0.644444444444444</v>
@@ -43418,7 +43632,7 @@
       </c>
       <c r="J32" s="38"/>
     </row>
-    <row r="33" ht="14.4" spans="1:10">
+    <row r="33" spans="1:10">
       <c r="A33" s="15">
         <v>30</v>
       </c>
@@ -43426,12 +43640,14 @@
         <v>46111</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D33" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="E33" s="19"/>
+      <c r="E33" s="17" t="s">
+        <v>195</v>
+      </c>
       <c r="F33" s="19"/>
       <c r="G33" s="40">
         <v>0.591666666666667</v>
@@ -43442,7 +43658,7 @@
       </c>
       <c r="J33" s="38"/>
     </row>
-    <row r="34" ht="14.4" spans="1:10">
+    <row r="34" spans="1:10">
       <c r="A34" s="17">
         <v>31</v>
       </c>
@@ -43450,12 +43666,14 @@
         <v>46112</v>
       </c>
       <c r="C34" s="30" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D34" s="19" t="s">
-        <v>143</v>
-      </c>
-      <c r="E34" s="19"/>
+        <v>173</v>
+      </c>
+      <c r="E34" s="17" t="s">
+        <v>196</v>
+      </c>
       <c r="F34" s="19"/>
       <c r="G34" s="40">
         <v>0.305555555555556</v>
@@ -44478,7 +44696,7 @@
       <c r="D2" s="5"/>
       <c r="E2" s="6"/>
       <c r="F2" s="7" t="s">
-        <v>145</v>
+        <v>197</v>
       </c>
       <c r="G2" s="8"/>
       <c r="H2" s="9" t="s">
@@ -44529,13 +44747,13 @@
         <v>46082</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D4" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F4" s="19"/>
       <c r="G4" s="20">
@@ -44555,13 +44773,13 @@
         <v>46083</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D5" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F5" s="23"/>
       <c r="G5" s="20">
@@ -44581,13 +44799,13 @@
         <v>46084</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D6" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F6" s="25"/>
       <c r="G6" s="20">
@@ -44607,13 +44825,13 @@
         <v>46085</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D7" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>147</v>
+        <v>199</v>
       </c>
       <c r="F7" s="27"/>
       <c r="G7" s="20">
@@ -44633,13 +44851,13 @@
         <v>46086</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D8" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>147</v>
+        <v>199</v>
       </c>
       <c r="F8" s="27"/>
       <c r="G8" s="20">
@@ -44659,13 +44877,13 @@
         <v>46087</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D9" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>147</v>
+        <v>199</v>
       </c>
       <c r="F9" s="27"/>
       <c r="G9" s="20">
@@ -44685,13 +44903,13 @@
         <v>46088</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D10" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>147</v>
+        <v>199</v>
       </c>
       <c r="F10" s="27"/>
       <c r="G10" s="20">
@@ -44711,13 +44929,13 @@
         <v>46089</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D11" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F11" s="27"/>
       <c r="G11" s="20">
@@ -44737,13 +44955,13 @@
         <v>46090</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D12" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F12" s="27"/>
       <c r="G12" s="20">
@@ -44763,13 +44981,13 @@
         <v>46091</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D13" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F13" s="27"/>
       <c r="G13" s="20">
@@ -44789,13 +45007,13 @@
         <v>46092</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D14" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F14" s="27"/>
       <c r="G14" s="20">
@@ -44815,13 +45033,13 @@
         <v>46093</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D15" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F15" s="27"/>
       <c r="G15" s="20">
@@ -44841,13 +45059,13 @@
         <v>46094</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D16" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F16" s="27"/>
       <c r="G16" s="28">
@@ -44867,13 +45085,13 @@
         <v>46095</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D17" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F17" s="27"/>
       <c r="G17" s="28">
@@ -44893,13 +45111,13 @@
         <v>46096</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D18" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F18" s="27"/>
       <c r="G18" s="28">
@@ -44919,13 +45137,13 @@
         <v>46097</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D19" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F19" s="27"/>
       <c r="G19" s="28">
@@ -44945,13 +45163,13 @@
         <v>46098</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D20" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F20" s="27"/>
       <c r="G20" s="20">
@@ -44971,13 +45189,13 @@
         <v>46099</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D21" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F21" s="27"/>
       <c r="G21" s="20">
@@ -44997,13 +45215,13 @@
         <v>46100</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D22" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F22" s="27"/>
       <c r="G22" s="20">
@@ -45023,13 +45241,13 @@
         <v>46101</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D23" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F23" s="27"/>
       <c r="G23" s="20">
@@ -45049,13 +45267,13 @@
         <v>46102</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D24" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F24" s="27"/>
       <c r="G24" s="20">
@@ -45075,13 +45293,13 @@
         <v>46103</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D25" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F25" s="27"/>
       <c r="G25" s="20">
@@ -45101,13 +45319,13 @@
         <v>46104</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D26" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F26" s="27"/>
       <c r="G26" s="20">
@@ -45127,13 +45345,13 @@
         <v>46105</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D27" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F27" s="27"/>
       <c r="G27" s="20">
@@ -45153,13 +45371,13 @@
         <v>46106</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D28" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E28" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F28" s="23"/>
       <c r="G28" s="20">
@@ -45179,13 +45397,13 @@
         <v>46107</v>
       </c>
       <c r="C29" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D29" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F29" s="27"/>
       <c r="G29" s="20">
@@ -45205,13 +45423,13 @@
         <v>46108</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D30" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F30" s="27"/>
       <c r="G30" s="20">
@@ -45231,13 +45449,13 @@
         <v>46109</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D31" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E31" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F31" s="23"/>
       <c r="G31" s="20">
@@ -45257,13 +45475,13 @@
         <v>46110</v>
       </c>
       <c r="C32" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D32" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F32" s="19"/>
       <c r="G32" s="20">
@@ -45283,13 +45501,13 @@
         <v>46111</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D33" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E33" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F33" s="19"/>
       <c r="G33" s="20">
@@ -45309,13 +45527,13 @@
         <v>46112</v>
       </c>
       <c r="C34" s="30" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="D34" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E34" s="18" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="F34" s="19"/>
       <c r="G34" s="20">

</xml_diff>